<commit_message>
Actualización documentación y evidencias
</commit_message>
<xml_diff>
--- a/docs/pruebas/casos_de_prueba.xlsx
+++ b/docs/pruebas/casos_de_prueba.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Odeth\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Corina\Desktop\ing\Joyería\docs\pruebas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB75826A-D30E-4964-AE4E-12E6B40220EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8195E111-F9C7-4000-84CD-395F572C9767}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82DA0B94-3521-42A6-9916-36604CCAD9CA}"/>
+    <workbookView xWindow="348" yWindow="348" windowWidth="4104" windowHeight="9696" xr2:uid="{82DA0B94-3521-42A6-9916-36604CCAD9CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos de prueba" sheetId="2" r:id="rId1"/>
@@ -23,12 +23,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="131">
   <si>
     <t>No</t>
   </si>
@@ -393,13 +387,52 @@
   </si>
   <si>
     <t>Consistencia de datos</t>
+  </si>
+  <si>
+    <t>Precondición</t>
+  </si>
+  <si>
+    <t>Pasos de ejecución</t>
+  </si>
+  <si>
+    <t>Resultado obtenido</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Sistema disponible y usuario con permisos correspondientes</t>
+  </si>
+  <si>
+    <t>Ejecutar acciones definidas y verificar comportamiento esperado</t>
+  </si>
+  <si>
+    <t>Coincide parcialmente con el resultado esperado</t>
+  </si>
+  <si>
+    <t>Aprobado</t>
+  </si>
+  <si>
+    <t>Con observaciones</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Observación</t>
+  </si>
+  <si>
+    <t>Cerrado (corregido)</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -419,8 +452,20 @@
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -433,13 +478,34 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -452,45 +518,64 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
+      <right/>
+      <top style="thin">
         <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF1155CC"/>
+      <color rgb="FF3333FF"/>
+      <color rgb="FF0066FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -819,15 +904,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57DCBE52-EBE4-4A03-A7B9-9AFFFEB7ECD1}">
-  <dimension ref="B2:G23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:M23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" customWidth="1"/>
-    <col min="5" max="6" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.59765625" customWidth="1"/>
+    <col min="4" max="4" width="15.09765625" customWidth="1"/>
+    <col min="5" max="6" width="14.69921875" customWidth="1"/>
+    <col min="8" max="8" width="18.296875" customWidth="1"/>
+    <col min="9" max="9" width="19.796875" customWidth="1"/>
+    <col min="10" max="10" width="19.296875" customWidth="1"/>
+    <col min="11" max="11" width="8.69921875" customWidth="1"/>
+    <col min="12" max="12" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" ht="31.2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -843,11 +933,29 @@
       <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="H2" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
@@ -866,8 +974,24 @@
       <c r="G3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H3" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K3" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M3" s="8"/>
+    </row>
+    <row r="4" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
@@ -886,8 +1010,24 @@
       <c r="G4" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K4" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M4" s="8"/>
+    </row>
+    <row r="5" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
@@ -906,8 +1046,24 @@
       <c r="G5" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" ht="78" x14ac:dyDescent="0.3">
+      <c r="H5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K5" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M5" s="8"/>
+    </row>
+    <row r="6" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
@@ -926,8 +1082,26 @@
       <c r="G6" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K6" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
@@ -946,8 +1120,26 @@
       <c r="G7" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K7" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
@@ -966,8 +1158,24 @@
       <c r="G8" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K8" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M8" s="9"/>
+    </row>
+    <row r="9" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>23</v>
       </c>
@@ -986,8 +1194,26 @@
       <c r="G9" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H9" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
@@ -1006,8 +1232,26 @@
       <c r="G10" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K10" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>28</v>
       </c>
@@ -1026,8 +1270,24 @@
       <c r="G11" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H11" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K11" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M11" s="8"/>
+    </row>
+    <row r="12" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
@@ -1046,8 +1306,24 @@
       <c r="G12" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K12" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M12" s="8"/>
+    </row>
+    <row r="13" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>34</v>
       </c>
@@ -1066,8 +1342,24 @@
       <c r="G13" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H13" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K13" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M13" s="8"/>
+    </row>
+    <row r="14" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>36</v>
       </c>
@@ -1086,28 +1378,60 @@
       <c r="G14" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="15" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B15" s="3" t="s">
+      <c r="H14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K14" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M14" s="8"/>
+    </row>
+    <row r="15" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K15" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M15" s="8"/>
+    </row>
+    <row r="16" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>41</v>
       </c>
@@ -1126,8 +1450,26 @@
       <c r="G16" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K16" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M16" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>45</v>
       </c>
@@ -1146,8 +1488,26 @@
       <c r="G17" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H17" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K17" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>46</v>
       </c>
@@ -1166,8 +1526,24 @@
       <c r="G18" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K18" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M18" s="8"/>
+    </row>
+    <row r="19" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>49</v>
       </c>
@@ -1186,8 +1562,26 @@
       <c r="G19" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="H19" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K19" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>53</v>
       </c>
@@ -1206,8 +1600,24 @@
       <c r="G20" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="21" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K20" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M20" s="8"/>
+    </row>
+    <row r="21" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>55</v>
       </c>
@@ -1226,8 +1636,24 @@
       <c r="G21" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="22" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K21" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M21" s="8"/>
+    </row>
+    <row r="22" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>58</v>
       </c>
@@ -1246,8 +1672,26 @@
       <c r="G22" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="23" spans="2:7" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="H22" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K22" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M22" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" ht="62.4" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
         <v>61</v>
       </c>
@@ -1265,6 +1709,24 @@
       </c>
       <c r="G23" s="2" t="s">
         <v>63</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K23" s="5">
+        <v>46143</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>